<commit_message>
Tables S11, S15, S16: rebuilt after the CPCT02010349T assignment change (code repo e6de415)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BtpRPVo656vetvDm7bkL5X
</commit_message>
<xml_diff>
--- a/sup_tables/sup_table_s15_sex_bias.xlsx
+++ b/sup_tables/sup_table_s15_sex_bias.xlsx
@@ -4103,223 +4103,223 @@
         <v>0.788592561767121</v>
       </c>
       <c r="H137" t="n">
-        <v>0.88577020415061</v>
+        <v>0.889831973119485</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="B138" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C138" t="s">
         <v>10</v>
       </c>
       <c r="D138" t="n">
-        <v>50</v>
+        <v>7</v>
       </c>
       <c r="E138" t="n">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="F138" t="n">
-        <v>0.676806064659977</v>
+        <v>0.621987350771959</v>
       </c>
       <c r="G138" t="n">
-        <v>1.16333561954796</v>
+        <v>1.27280000664737</v>
       </c>
       <c r="H138" t="n">
-        <v>0.88577020415061</v>
+        <v>0.889831973119485</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="B139" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C139" t="s">
         <v>10</v>
       </c>
       <c r="D139" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E139" t="n">
-        <v>144</v>
+        <v>91</v>
       </c>
       <c r="F139" t="n">
-        <v>0.682766935282337</v>
+        <v>0.61523915372729</v>
       </c>
       <c r="G139" t="n">
-        <v>0.829147013792629</v>
+        <v>1.33402615134227</v>
       </c>
       <c r="H139" t="n">
-        <v>0.88577020415061</v>
+        <v>0.889831973119485</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B140" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="C140" t="s">
         <v>10</v>
       </c>
       <c r="D140" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="E140" t="n">
-        <v>25</v>
+        <v>88</v>
       </c>
       <c r="F140" t="n">
-        <v>0.621987350771959</v>
+        <v>0.662281264954675</v>
       </c>
       <c r="G140" t="n">
-        <v>1.27280000664737</v>
+        <v>0.854942528910744</v>
       </c>
       <c r="H140" t="n">
-        <v>0.88577020415061</v>
+        <v>0.889831973119485</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="B141" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="C141" t="s">
         <v>10</v>
       </c>
       <c r="D141" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E141" t="n">
-        <v>91</v>
+        <v>18</v>
       </c>
       <c r="F141" t="n">
-        <v>0.61523915372729</v>
+        <v>0.637077147527254</v>
       </c>
       <c r="G141" t="n">
-        <v>1.33402615134227</v>
+        <v>0.722902475292088</v>
       </c>
       <c r="H141" t="n">
-        <v>0.88577020415061</v>
+        <v>0.889831973119485</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="B142" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C142" t="s">
         <v>10</v>
       </c>
       <c r="D142" t="n">
-        <v>70</v>
+        <v>9</v>
       </c>
       <c r="E142" t="n">
-        <v>44</v>
+        <v>81</v>
       </c>
       <c r="F142" t="n">
-        <v>0.703405750354896</v>
+        <v>0.651409377460877</v>
       </c>
       <c r="G142" t="n">
-        <v>1.10385314529785</v>
+        <v>0.753251838544302</v>
       </c>
       <c r="H142" t="n">
-        <v>0.88577020415061</v>
+        <v>0.889831973119485</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B143" t="s">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="C143" t="s">
         <v>10</v>
       </c>
       <c r="D143" t="n">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="E143" t="n">
-        <v>71</v>
+        <v>143</v>
       </c>
       <c r="F143" t="n">
-        <v>0.695484616740845</v>
+        <v>0.663012058402754</v>
       </c>
       <c r="G143" t="n">
-        <v>1.1380145178319</v>
+        <v>1.16494331419245</v>
       </c>
       <c r="H143" t="n">
-        <v>0.88577020415061</v>
+        <v>0.889831973119485</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="B144" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="C144" t="s">
         <v>10</v>
       </c>
       <c r="D144" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="E144" t="n">
-        <v>88</v>
+        <v>168</v>
       </c>
       <c r="F144" t="n">
-        <v>0.662281264954675</v>
+        <v>0.589042267367359</v>
       </c>
       <c r="G144" t="n">
-        <v>0.854942528910744</v>
+        <v>1.24802574892841</v>
       </c>
       <c r="H144" t="n">
-        <v>0.88577020415061</v>
+        <v>0.896491338288336</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="B145" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="C145" t="s">
         <v>10</v>
       </c>
       <c r="D145" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E145" t="n">
-        <v>18</v>
+        <v>91</v>
       </c>
       <c r="F145" t="n">
-        <v>0.637077147527254</v>
+        <v>0.61523915372729</v>
       </c>
       <c r="G145" t="n">
-        <v>0.722902475292088</v>
+        <v>1.33402615134227</v>
       </c>
       <c r="H145" t="n">
-        <v>0.88577020415061</v>
+        <v>0.896491338288336</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="B146" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C146" t="s">
         <v>10</v>
@@ -4328,16 +4328,16 @@
         <v>9</v>
       </c>
       <c r="E146" t="n">
-        <v>81</v>
+        <v>25</v>
       </c>
       <c r="F146" t="n">
-        <v>0.651409377460877</v>
+        <v>0.60960398069094</v>
       </c>
       <c r="G146" t="n">
-        <v>0.753251838544302</v>
+        <v>0.695857133745228</v>
       </c>
       <c r="H146" t="n">
-        <v>0.88577020415061</v>
+        <v>0.896491338288336</v>
       </c>
     </row>
     <row r="147">
@@ -4345,207 +4345,207 @@
         <v>8</v>
       </c>
       <c r="B147" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="C147" t="s">
         <v>10</v>
       </c>
       <c r="D147" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="E147" t="n">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="F147" t="n">
-        <v>0.663012058402754</v>
+        <v>0.615173320702119</v>
       </c>
       <c r="G147" t="n">
-        <v>1.16494331419245</v>
+        <v>1.13741434866417</v>
       </c>
       <c r="H147" t="n">
-        <v>0.88577020415061</v>
+        <v>0.896491338288336</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>8</v>
+        <v>38</v>
       </c>
       <c r="B148" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="C148" t="s">
         <v>10</v>
       </c>
       <c r="D148" t="n">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="E148" t="n">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="F148" t="n">
-        <v>0.699179681198832</v>
+        <v>0.682766935282337</v>
       </c>
       <c r="G148" t="n">
-        <v>1.12799460199462</v>
+        <v>0.829147013792629</v>
       </c>
       <c r="H148" t="n">
-        <v>0.88577020415061</v>
+        <v>0.896842331702493</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="B149" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="C149" t="s">
         <v>10</v>
       </c>
       <c r="D149" t="n">
-        <v>17</v>
+        <v>70</v>
       </c>
       <c r="E149" t="n">
-        <v>73</v>
+        <v>44</v>
       </c>
       <c r="F149" t="n">
-        <v>0.719823508255764</v>
+        <v>0.703405750354896</v>
       </c>
       <c r="G149" t="n">
-        <v>0.837021648649028</v>
+        <v>1.10385314529785</v>
       </c>
       <c r="H149" t="n">
-        <v>0.895390217586438</v>
+        <v>0.896842331702493</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="B150" t="s">
-        <v>63</v>
+        <v>24</v>
       </c>
       <c r="C150" t="s">
         <v>10</v>
       </c>
       <c r="D150" t="n">
-        <v>16</v>
+        <v>43</v>
       </c>
       <c r="E150" t="n">
-        <v>168</v>
+        <v>71</v>
       </c>
       <c r="F150" t="n">
-        <v>0.589042267367359</v>
+        <v>0.695484616740845</v>
       </c>
       <c r="G150" t="n">
-        <v>1.24802574892841</v>
+        <v>1.1380145178319</v>
       </c>
       <c r="H150" t="n">
-        <v>0.896491338288336</v>
+        <v>0.896842331702493</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="B151" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C151" t="s">
         <v>10</v>
       </c>
       <c r="D151" t="n">
-        <v>7</v>
+        <v>36</v>
       </c>
       <c r="E151" t="n">
-        <v>91</v>
+        <v>134</v>
       </c>
       <c r="F151" t="n">
-        <v>0.61523915372729</v>
+        <v>0.699179681198832</v>
       </c>
       <c r="G151" t="n">
-        <v>1.33402615134227</v>
+        <v>1.12799460199462</v>
       </c>
       <c r="H151" t="n">
-        <v>0.896491338288336</v>
+        <v>0.896842331702493</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="B152" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="C152" t="s">
         <v>10</v>
       </c>
       <c r="D152" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="E152" t="n">
-        <v>25</v>
+        <v>73</v>
       </c>
       <c r="F152" t="n">
-        <v>0.60960398069094</v>
+        <v>0.719823508255764</v>
       </c>
       <c r="G152" t="n">
-        <v>0.695857133745228</v>
+        <v>0.837021648649028</v>
       </c>
       <c r="H152" t="n">
-        <v>0.896491338288336</v>
+        <v>0.906444417803554</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B153" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C153" t="s">
         <v>10</v>
       </c>
       <c r="D153" t="n">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="E153" t="n">
-        <v>132</v>
+        <v>94</v>
       </c>
       <c r="F153" t="n">
-        <v>0.615173320702119</v>
+        <v>0.739905876333053</v>
       </c>
       <c r="G153" t="n">
-        <v>1.13741434866417</v>
+        <v>1.11884130194171</v>
       </c>
       <c r="H153" t="n">
-        <v>0.896491338288336</v>
+        <v>0.90942505050934</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B154" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="C154" t="s">
         <v>10</v>
       </c>
       <c r="D154" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E154" t="n">
-        <v>94</v>
+        <v>153</v>
       </c>
       <c r="F154" t="n">
-        <v>0.739905876333053</v>
+        <v>0.740022345022306</v>
       </c>
       <c r="G154" t="n">
-        <v>1.11884130194171</v>
+        <v>0.852211314182209</v>
       </c>
       <c r="H154" t="n">
-        <v>0.8985985618128</v>
+        <v>0.90942505050934</v>
       </c>
     </row>
     <row r="155">
@@ -4553,30 +4553,30 @@
         <v>8</v>
       </c>
       <c r="B155" t="s">
-        <v>56</v>
+        <v>24</v>
       </c>
       <c r="C155" t="s">
         <v>10</v>
       </c>
       <c r="D155" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="E155" t="n">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="F155" t="n">
-        <v>0.740022345022306</v>
+        <v>0.752386008643869</v>
       </c>
       <c r="G155" t="n">
-        <v>0.852211314182209</v>
+        <v>1.13924181298246</v>
       </c>
       <c r="H155" t="n">
-        <v>0.8985985618128</v>
+        <v>0.913611581924698</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="B156" t="s">
         <v>24</v>
@@ -4585,19 +4585,19 @@
         <v>10</v>
       </c>
       <c r="D156" t="n">
-        <v>22</v>
+        <v>49</v>
       </c>
       <c r="E156" t="n">
-        <v>148</v>
+        <v>54</v>
       </c>
       <c r="F156" t="n">
-        <v>0.752386008643869</v>
+        <v>0.780964594546653</v>
       </c>
       <c r="G156" t="n">
-        <v>1.13924181298246</v>
+        <v>1.11916834550915</v>
       </c>
       <c r="H156" t="n">
-        <v>0.902863210372642</v>
+        <v>0.934553588600633</v>
       </c>
     </row>
     <row r="157">

</xml_diff>